<commit_message>
Add unit tests for various helpers, middleware, and routes >> >> - Implement tests for value helper functions including isEmpty, isNumeric, isJson, isDomainAddress, randomString, maskSensitiveData, excelColumnName, and safeJsonParse. >> - Create tests for authentication middleware functions: authenticateToken, authenticateRefreshToken, and authenticateKey. >> - Add tests for entities, exports, FAQ answers, FAQ questions, FAQs, files, languages, token, users, and webhook routes. >> - Mock necessary dependencies and ensure proper request handling in tests. >> - Update TypeScript configuration to include test files and add types for node, jest, and multer.
</commit_message>
<xml_diff>
--- a/public/template-entities.xlsx
+++ b/public/template-entities.xlsx
@@ -1,10 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
-  <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B61B7F2-8913-4C5F-BC68-A05A0C86C8D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="16392" windowHeight="6036"/>
+    <workbookView xWindow="-23385" yWindow="6375" windowWidth="17280" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
@@ -14,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="28">
   <si>
     <t>Intent</t>
   </si>
@@ -26,12 +27,84 @@
   </si>
   <si>
     <t>Aliases</t>
+  </si>
+  <si>
+    <t>greeting</t>
+  </si>
+  <si>
+    <t>day</t>
+  </si>
+  <si>
+    <t>store</t>
+  </si>
+  <si>
+    <t>location</t>
+  </si>
+  <si>
+    <t>halo</t>
+  </si>
+  <si>
+    <t>pagi</t>
+  </si>
+  <si>
+    <t>siang</t>
+  </si>
+  <si>
+    <t>sore</t>
+  </si>
+  <si>
+    <t>malam</t>
+  </si>
+  <si>
+    <t>toko</t>
+  </si>
+  <si>
+    <t>warung</t>
+  </si>
+  <si>
+    <t>tempat makan</t>
+  </si>
+  <si>
+    <t>alamat</t>
+  </si>
+  <si>
+    <t>lokasi</t>
+  </si>
+  <si>
+    <t>id</t>
+  </si>
+  <si>
+    <t>helo, hai, test</t>
+  </si>
+  <si>
+    <t>pagii, subuh</t>
+  </si>
+  <si>
+    <t>siaang</t>
+  </si>
+  <si>
+    <t>petang</t>
+  </si>
+  <si>
+    <t>tokonya</t>
+  </si>
+  <si>
+    <t>warungnya</t>
+  </si>
+  <si>
+    <t>tempatmakan, restoran</t>
+  </si>
+  <si>
+    <t>alamatnya</t>
+  </si>
+  <si>
+    <t>lokasinya</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -384,8 +457,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:D11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="4" width="20.77734375" customWidth="1"/>
@@ -405,6 +478,143 @@
         <v>3</v>
       </c>
     </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D7" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" t="s">
+        <v>18</v>
+      </c>
+      <c r="D8" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>6</v>
+      </c>
+      <c r="B9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D9" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>7</v>
+      </c>
+      <c r="B10" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>7</v>
+      </c>
+      <c r="B11" t="s">
+        <v>17</v>
+      </c>
+      <c r="C11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11" t="s">
+        <v>27</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>